<commit_message>
templates: fixed-asset register 2026-08-24 (verified, 41 checks, 2d9e7fe26cdcebaa)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/smbsolved-fixed-asset-register.xlsx
+++ b/templates/smbsolved-fixed-asset-register.xlsx
@@ -2,26 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\smbsolved-marketing\out\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5DF2E03C-4C0E-434F-843B-EE74B943DCC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34181220-C944-4F26-B1E9-F2FDDDEA43E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-31950" yWindow="2415" windowWidth="24885" windowHeight="17775" activeTab="2" xr2:uid="{81740E39-A5A5-4EE9-9693-464C971E4014}"/>
+    <workbookView xWindow="2655" yWindow="2835" windowWidth="34845" windowHeight="17775" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
     <sheet name="Register" sheetId="2" r:id="rId2"/>
     <sheet name="Readme" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -33,37 +30,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
+    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="67">
   <si>
     <t>MACRS GDS, half-year convention (200% DB; 15-year is 150% DB)</t>
   </si>
@@ -74,9 +49,6 @@
     <t>FIXED ASSET REGISTER &amp; ROLL-FORWARD</t>
   </si>
   <si>
-    <t>smbsolved.com Â· every formula verified in real Excel Â· yellow cells are inputs</t>
-  </si>
-  <si>
     <t>Report year</t>
   </si>
   <si>
@@ -155,6 +127,12 @@
     <t>_disp</t>
   </si>
   <si>
+    <t>Check</t>
+  </si>
+  <si>
+    <t>_prior</t>
+  </si>
+  <si>
     <t>FA-0001</t>
   </si>
   <si>
@@ -218,6 +196,9 @@
     <t>Net book value</t>
   </si>
   <si>
+    <t>Input check</t>
+  </si>
+  <si>
     <t>TIE TO GL</t>
   </si>
   <si>
@@ -239,19 +220,25 @@
     <t>Tax depreciation is MACRS GDS half-year (percentages on the Tables sheet). Bonus % applies in year one and reduces the MACRS basis. Section 179 is not modeled; ask your tax preparer.</t>
   </si>
   <si>
+    <t>The Check column flags bad inputs row by row, and the Input check line under the roll-forward counts how many rows need attention. Both should read OK.</t>
+  </si>
+  <si>
     <t>The tie-out rows should read OK. If one shows a number, that number is exactly how far off you are.</t>
   </si>
   <si>
-    <t>Remove assets disposed of in years before the report year; the register shows the current year only.</t>
-  </si>
-  <si>
-    <t>Add rows: insert above the TOTALS row, then fill the formulas down from the row above.</t>
+    <t>Assets disposed of in a year before the report year carry no cost and no accumulated depreciation, so the roll-forward still ties. The Check column will tell you to remove the row.</t>
+  </si>
+  <si>
+    <t>Add rows: insert above the TOTALS row, then fill the formulas down from the row above. Extend the SUM and SUMPRODUCT ranges in the totals and roll-forward to cover the new rows.</t>
+  </si>
+  <si>
+    <t>Tax classes supported: 3, 5, 7, 10 and 15 year. Real property (20, 27.5 and 39 year) uses a mid-month convention and is not modeled.</t>
+  </si>
+  <si>
+    <t>Columns X, Y and AA are hidden helper flags. Leave them alone.</t>
   </si>
   <si>
     <t>No macros. Works in Excel 2016 and later.</t>
-  </si>
-  <si>
-    <t>Every formula in this file was computed and checked in real Excel before publishing.</t>
   </si>
 </sst>
 </file>
@@ -264,7 +251,22 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF5A5A5A"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <b/>
@@ -272,25 +274,10 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF5A5A5A"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -300,7 +287,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF99"/>
-        <bgColor indexed="64"/>
+        <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -316,24 +309,244 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="4" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="22">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFCC"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFCC"/>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFCC"/>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFCC"/>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFCC"/>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFCC"/>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFCC"/>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFCC"/>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFCC"/>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFCC"/>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFCC"/>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF5A5A5A"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -345,15 +558,82 @@
 </styleSheet>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B14C5D2E-EB63-4F09-AD2E-1FA5E95DA8BA}" name="Table1" displayName="Table1" ref="A4:Z10" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A4:Z10" xr:uid="{B14C5D2E-EB63-4F09-AD2E-1FA5E95DA8BA}"/>
+  <tableColumns count="26">
+    <tableColumn id="1" xr3:uid="{CBF54419-F41E-48DE-B9BB-B6031C1C6D33}" name="Asset ID" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{3DAB9C72-A257-43F3-84B3-C329822A363D}" name="Description" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{1149EF4C-BE9F-47E5-9742-1015D944387C}" name="In service" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{900A4B1D-4C17-4888-96BC-DBF8F88C4484}" name="Cost" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{38DCB2E2-46D1-44D9-98C3-34F1A6E2A2A0}" name="Salvage" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{5209CEFD-123D-4913-AC7D-CB5C3ED2AE7A}" name="Life (yrs)" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{A8E1B157-E04E-4CD4-A3E8-21B82EA76DBA}" name="Tax class" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{8892CD50-1877-4DEA-A50C-A86E1EF2D2B5}" name="Bonus %" dataDxfId="14"/>
+    <tableColumn id="9" xr3:uid="{FEDCCE52-DF00-4A14-82D9-0288B7479BB4}" name="Disposed" dataDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{AD73CCA0-FDA1-49DE-887D-A17A5301FDC3}" name="Proceeds" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{D6DF66AD-D40D-4D29-8447-21727AA0D8B2}" name="Mo. prior">
+      <calculatedColumnFormula>IF($C5="","",MAX(0,MIN($F5*12,($B$3-1-YEAR($C5))*12+13-MONTH($C5))))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="12" xr3:uid="{7ADC367C-21E9-41B3-BDA1-73A742028056}" name="Mo. this yr">
+      <calculatedColumnFormula>IF($C5="","",IF(YEAR($C5)&gt;$B$3,0,IF(AND($I5&lt;&gt;"",YEAR($I5)&lt;$B$3),0,MAX(0,MIN(IF(AND($I5&lt;&gt;"",YEAR($I5)=$B$3),MONTH($I5)-1,12)-IF(YEAR($C5)=$B$3,MONTH($C5),1)+1,$F5*12-K5)))))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="13" xr3:uid="{BE403D8F-C98B-4DA8-9628-301FAE257EA9}" name="Monthly dep" dataDxfId="11">
+      <calculatedColumnFormula>IF($C5="","",IF($F5&gt;0,MAX(0,$D5-$E5)/($F5*12),0))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="14" xr3:uid="{4CCF4246-837D-4F75-80D2-DA4FC600D166}" name="Beg A/D" dataDxfId="10">
+      <calculatedColumnFormula>IF($C5="","",IF($AA5=1,0,K5*M5))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="15" xr3:uid="{BADDA35B-F607-4B4D-BB62-BA436E45B912}" name="Dep this yr" dataDxfId="9">
+      <calculatedColumnFormula>IF($C5="","",L5*M5)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="16" xr3:uid="{123857C0-9B04-46E2-A418-4BE7006ECD81}" name="A/D relieved" dataDxfId="8">
+      <calculatedColumnFormula>IF($C5="",0,IF(Y5=1,N5+O5,0))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="17" xr3:uid="{8304A90D-F555-499C-822E-04611BD28634}" name="End A/D" dataDxfId="7">
+      <calculatedColumnFormula>IF($C5="","",IF(OR(Y5=1,$AA5=1),0,N5+O5))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="18" xr3:uid="{8B576254-2490-4600-B259-97AF59E98114}" name="End cost" dataDxfId="6">
+      <calculatedColumnFormula>IF($C5="","",IF(OR(Y5=1,AND($I5&lt;&gt;"",YEAR($I5)&lt;$B$3)),0,$D5))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="19" xr3:uid="{287B67CB-FEB0-435B-B3F7-698CDBF6D95D}" name="NBV" dataDxfId="5">
+      <calculatedColumnFormula>IF($C5="","",R5-Q5)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="20" xr3:uid="{4396BFAB-CF90-4CB7-8E34-74F4AB7C10EB}" name="Gain/(loss)" dataDxfId="4">
+      <calculatedColumnFormula>IF(Y5=1,$J5-($D5-P5),"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="21" xr3:uid="{2CEA2750-8FA0-4360-92D0-128C28E5573E}" name="Tax yr">
+      <calculatedColumnFormula>IF($C5="","",$B$3-YEAR($C5)+1)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="22" xr3:uid="{590E8150-E959-4632-B460-9398286E3038}" name="MACRS %" dataDxfId="3">
+      <calculatedColumnFormula>IF($C5="","",IF(U5&lt;1,0,IFERROR(INDEX(Tables!$B$3:$F$18,U5,MATCH($G5,Tables!$B$2:$F$2,0)),0)))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="23" xr3:uid="{8594DEDF-0340-4608-B861-E89FA7CFA0E5}" name="Tax dep" dataDxfId="2">
+      <calculatedColumnFormula>IF($C5="","",IF(OR($AA5=1,YEAR($C5)&gt;$B$3),0,($D5*(1-$H5))*V5*IF(Y5=1,0.5,1)+IF(U5=1,$D5*$H5,0)))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="24" xr3:uid="{D93EDCB3-E185-48B5-9749-9AC9D4198532}" name="_add">
+      <calculatedColumnFormula>IF($C5="",0,IF(YEAR($C5)=$B$3,1,0))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="25" xr3:uid="{75205E7A-07DE-4C28-8F53-708F58A2F956}" name="_disp">
+      <calculatedColumnFormula>IF($C5="",0,IF(AND($I5&lt;&gt;"",YEAR($I5)=$B$3),1,0))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="26" xr3:uid="{12ECB5F9-C916-4EDD-BF89-543CCDB4A272}" name="Check" dataDxfId="0">
+      <calculatedColumnFormula>IF($C5="","",IF($F5&lt;=0,"Life must be greater than 0",IF($D5&lt;0,"Cost cannot be negative",IF($E5&gt;$D5,"Salvage exceeds cost",IF(YEAR($C5)&gt;$B$3,"In-service date is after the report year",IF(AND($I5&lt;&gt;"",$I5&lt;$C5),"Disposal date is before in-service date",IF(ISNA(MATCH($G5,Tables!$B$2:$F$2,0)),"Tax class must be 3, 5, 7, 10 or 15",IF($AA5=1,"Disposed in a prior year - remove this row","OK"))))))))</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -391,150 +671,52 @@
         <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme>
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
                 <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
                 <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
                 <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
                 <a:lumMod val="102000"/>
                 <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
                 <a:lumMod val="100000"/>
                 <a:shade val="100000"/>
               </a:schemeClr>
@@ -542,33 +724,24 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
                 <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
@@ -581,13 +754,7 @@
           <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -597,15 +764,13 @@
         <a:solidFill>
           <a:schemeClr val="phClr">
             <a:tint val="95000"/>
-            <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
               </a:schemeClr>
@@ -613,7 +778,6 @@
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
               </a:schemeClr>
@@ -621,56 +785,31 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="63000"/>
-                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80E6F944-92A0-45CA-AB81-D7301A1E4ACC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F18"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -690,7 +829,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -710,7 +849,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -730,7 +869,7 @@
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -750,7 +889,7 @@
         <v>8.5500000000000007E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -770,7 +909,7 @@
         <v>7.6999999999999999E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -788,7 +927,7 @@
         <v>6.93E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -806,7 +945,7 @@
         <v>6.2300000000000001E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -822,7 +961,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -838,7 +977,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -852,7 +991,7 @@
         <v>5.91E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
@@ -866,7 +1005,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -880,7 +1019,7 @@
         <v>5.91E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -892,7 +1031,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
@@ -904,7 +1043,7 @@
         <v>5.91E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>
@@ -916,7 +1055,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
@@ -928,7 +1067,7 @@
         <v>5.91E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>16</v>
       </c>
@@ -941,121 +1080,131 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5238526F-181E-4A29-A33E-645525A16F11}">
-  <dimension ref="A1:Y25"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:AA25"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.7109375" customWidth="1"/>
-    <col min="3" max="23" width="12.7109375" customWidth="1"/>
-    <col min="24" max="25" width="0" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="12" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="12.85546875" customWidth="1"/>
+    <col min="14" max="23" width="12.7109375" customWidth="1"/>
+    <col min="24" max="25" width="10.140625" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="11.42578125" customWidth="1"/>
+    <col min="27" max="27" width="13" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:27" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:27" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3"/>
+    </row>
+    <row r="3" spans="1:27" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" s="4">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" s="12" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="5">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="B4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="J4" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="L4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="M4" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="N4" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="O4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="P4" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="Q4" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="R4" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="S4" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="S4" s="2" t="s">
+      <c r="T4" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="T4" s="2" t="s">
+      <c r="U4" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="U4" s="2" t="s">
+      <c r="V4" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="V4" s="2" t="s">
+      <c r="W4" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="W4" s="2" t="s">
+      <c r="X4" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="X4" s="2" t="s">
+      <c r="Y4" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="Y4" s="2" t="s">
+      <c r="Z4" s="11" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="AA4" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="5" t="s">
+    </row>
+    <row r="5" spans="1:27" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>31</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>32</v>
       </c>
       <c r="C5" s="6">
         <v>45000</v>
@@ -1066,84 +1215,92 @@
       <c r="E5" s="7">
         <v>2500</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="4">
         <v>7</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="4">
         <v>5</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H5" s="8">
         <v>0</v>
       </c>
       <c r="I5" s="6"/>
       <c r="J5" s="7"/>
       <c r="K5">
-        <f>IF($C5="","",MAX(0,MIN($F5*12,($B$3-1-YEAR($C5))*12+13-MONTH($C5))))</f>
+        <f t="shared" ref="K5:K10" si="0">IF($C5="","",MAX(0,MIN($F5*12,($B$3-1-YEAR($C5))*12+13-MONTH($C5))))</f>
         <v>34</v>
       </c>
       <c r="L5">
-        <f>IF($C5="","",IF(YEAR($C5)&gt;$B$3,0,IF(AND($I5&lt;&gt;"",YEAR($I5)&lt;$B$3),0,MAX(0,MIN(IF(AND($I5&lt;&gt;"",YEAR($I5)=$B$3),MONTH($I5)-1,12)-IF(YEAR($C5)=$B$3,MONTH($C5),1)+1,$F5*12-K5)))))</f>
+        <f t="shared" ref="L5:L10" si="1">IF($C5="","",IF(YEAR($C5)&gt;$B$3,0,IF(AND($I5&lt;&gt;"",YEAR($I5)&lt;$B$3),0,MAX(0,MIN(IF(AND($I5&lt;&gt;"",YEAR($I5)=$B$3),MONTH($I5)-1,12)-IF(YEAR($C5)=$B$3,MONTH($C5),1)+1,$F5*12-K5)))))</f>
         <v>12</v>
       </c>
       <c r="M5" s="9">
-        <f>IF($C5="","",($D5-$E5)/($F5*12))</f>
+        <f t="shared" ref="M5:M10" si="2">IF($C5="","",IF($F5&gt;0,MAX(0,$D5-$E5)/($F5*12),0))</f>
         <v>309.52380952380952</v>
       </c>
       <c r="N5" s="9">
-        <f>IF($C5="","",K5*M5)</f>
+        <f t="shared" ref="N5:N10" si="3">IF($C5="","",IF($AA5=1,0,K5*M5))</f>
         <v>10523.809523809523</v>
       </c>
       <c r="O5" s="9">
-        <f>IF($C5="","",L5*M5)</f>
+        <f t="shared" ref="O5:O10" si="4">IF($C5="","",L5*M5)</f>
         <v>3714.2857142857142</v>
       </c>
       <c r="P5" s="9">
-        <f>IF(Y5=1,N5+O5,0)</f>
+        <f t="shared" ref="P5:P10" si="5">IF($C5="",0,IF(Y5=1,N5+O5,0))</f>
         <v>0</v>
       </c>
       <c r="Q5" s="9">
-        <f>IF($C5="","",IF(Y5=1,0,N5+O5))</f>
+        <f t="shared" ref="Q5:Q10" si="6">IF($C5="","",IF(OR(Y5=1,$AA5=1),0,N5+O5))</f>
         <v>14238.095238095237</v>
       </c>
       <c r="R5" s="9">
-        <f>IF($C5="","",IF(OR(Y5=1,AND($I5&lt;&gt;"",YEAR($I5)&lt;$B$3)),0,$D5))</f>
+        <f t="shared" ref="R5:R10" si="7">IF($C5="","",IF(OR(Y5=1,AND($I5&lt;&gt;"",YEAR($I5)&lt;$B$3)),0,$D5))</f>
         <v>28500</v>
       </c>
       <c r="S5" s="9">
-        <f>IF($C5="","",R5-Q5)</f>
+        <f t="shared" ref="S5:S10" si="8">IF($C5="","",R5-Q5)</f>
         <v>14261.904761904763</v>
       </c>
       <c r="T5" s="9" t="str">
-        <f>IF(Y5=1,$J5-($D5-P5),"")</f>
+        <f t="shared" ref="T5:T10" si="9">IF(Y5=1,$J5-($D5-P5),"")</f>
         <v/>
       </c>
       <c r="U5">
-        <f>IF($C5="","",$B$3-YEAR($C5)+1)</f>
+        <f t="shared" ref="U5:U10" si="10">IF($C5="","",$B$3-YEAR($C5)+1)</f>
         <v>4</v>
       </c>
-      <c r="V5" s="1" cm="1">
-        <f t="array" ref="V5">IF($C5="","",IFERROR(INDEX(Tables!$B$3:$F$18,U5,MATCH($G5,Tables!$B$2:$F$2,0)),0))</f>
+      <c r="V5" s="1">
+        <f>IF($C5="","",IF(U5&lt;1,0,IFERROR(INDEX(Tables!$B$3:$F$18,U5,MATCH($G5,Tables!$B$2:$F$2,0)),0)))</f>
         <v>0.1152</v>
       </c>
       <c r="W5" s="9">
-        <f>IF($C5="","",IF(AND($I5&lt;&gt;"",YEAR($I5)&lt;$B$3),0,($D5*(1-$H5))*V5*IF(Y5=1,0.5,1)+IF(U5=1,$D5*$H5,0)))</f>
+        <f t="shared" ref="W5:W10" si="11">IF($C5="","",IF(OR($AA5=1,YEAR($C5)&gt;$B$3),0,($D5*(1-$H5))*V5*IF(Y5=1,0.5,1)+IF(U5=1,$D5*$H5,0)))</f>
         <v>3283.2</v>
       </c>
       <c r="X5">
-        <f>IF($C5="",0,IF(YEAR($C5)=$B$3,1,0))</f>
+        <f t="shared" ref="X5:X10" si="12">IF($C5="",0,IF(YEAR($C5)=$B$3,1,0))</f>
         <v>0</v>
       </c>
       <c r="Y5">
-        <f>IF($C5="",0,IF(AND($I5&lt;&gt;"",YEAR($I5)=$B$3),1,0))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="5" t="s">
+        <f t="shared" ref="Y5:Y10" si="13">IF($C5="",0,IF(AND($I5&lt;&gt;"",YEAR($I5)=$B$3),1,0))</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="13" t="str">
+        <f>IF($C5="","",IF($F5&lt;=0,"Life must be greater than 0",IF($D5&lt;0,"Cost cannot be negative",IF($E5&gt;$D5,"Salvage exceeds cost",IF(YEAR($C5)&gt;$B$3,"In-service date is after the report year",IF(AND($I5&lt;&gt;"",$I5&lt;$C5),"Disposal date is before in-service date",IF(ISNA(MATCH($G5,Tables!$B$2:$F$2,0)),"Tax class must be 3, 5, 7, 10 or 15",IF($AA5=1,"Disposed in a prior year - remove this row","OK"))))))))</f>
+        <v>OK</v>
+      </c>
+      <c r="AA5" s="4">
+        <f t="shared" ref="AA5:AA10" si="14">IF($C5="",0,IF(AND($I5&lt;&gt;"",YEAR($I5)&lt;$B$3),1,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>33</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>34</v>
       </c>
       <c r="C6" s="6">
         <v>45474</v>
@@ -1154,84 +1311,92 @@
       <c r="E6" s="7">
         <v>0</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="4">
         <v>10</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="4">
         <v>15</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6" s="8">
         <v>0</v>
       </c>
       <c r="I6" s="6"/>
       <c r="J6" s="7"/>
       <c r="K6">
-        <f>IF($C6="","",MAX(0,MIN($F6*12,($B$3-1-YEAR($C6))*12+13-MONTH($C6))))</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="L6">
-        <f>IF($C6="","",IF(YEAR($C6)&gt;$B$3,0,IF(AND($I6&lt;&gt;"",YEAR($I6)&lt;$B$3),0,MAX(0,MIN(IF(AND($I6&lt;&gt;"",YEAR($I6)=$B$3),MONTH($I6)-1,12)-IF(YEAR($C6)=$B$3,MONTH($C6),1)+1,$F6*12-K6)))))</f>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="M6" s="9">
-        <f>IF($C6="","",($D6-$E6)/($F6*12))</f>
+        <f t="shared" si="2"/>
         <v>535</v>
       </c>
       <c r="N6" s="9">
-        <f>IF($C6="","",K6*M6)</f>
+        <f t="shared" si="3"/>
         <v>9630</v>
       </c>
       <c r="O6" s="9">
-        <f>IF($C6="","",L6*M6)</f>
+        <f t="shared" si="4"/>
         <v>6420</v>
       </c>
       <c r="P6" s="9">
-        <f>IF(Y6=1,N6+O6,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Q6" s="9">
-        <f>IF($C6="","",IF(Y6=1,0,N6+O6))</f>
+        <f t="shared" si="6"/>
         <v>16050</v>
       </c>
       <c r="R6" s="9">
-        <f>IF($C6="","",IF(OR(Y6=1,AND($I6&lt;&gt;"",YEAR($I6)&lt;$B$3)),0,$D6))</f>
+        <f t="shared" si="7"/>
         <v>64200</v>
       </c>
       <c r="S6" s="9">
-        <f>IF($C6="","",R6-Q6)</f>
+        <f t="shared" si="8"/>
         <v>48150</v>
       </c>
       <c r="T6" s="9" t="str">
-        <f>IF(Y6=1,$J6-($D6-P6),"")</f>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="U6">
-        <f>IF($C6="","",$B$3-YEAR($C6)+1)</f>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
-      <c r="V6" s="1" cm="1">
-        <f t="array" ref="V6">IF($C6="","",IFERROR(INDEX(Tables!$B$3:$F$18,U6,MATCH($G6,Tables!$B$2:$F$2,0)),0))</f>
+      <c r="V6" s="1">
+        <f>IF($C6="","",IF(U6&lt;1,0,IFERROR(INDEX(Tables!$B$3:$F$18,U6,MATCH($G6,Tables!$B$2:$F$2,0)),0)))</f>
         <v>8.5500000000000007E-2</v>
       </c>
       <c r="W6" s="9">
-        <f>IF($C6="","",IF(AND($I6&lt;&gt;"",YEAR($I6)&lt;$B$3),0,($D6*(1-$H6))*V6*IF(Y6=1,0.5,1)+IF(U6=1,$D6*$H6,0)))</f>
+        <f t="shared" si="11"/>
         <v>5489.1</v>
       </c>
       <c r="X6">
-        <f>IF($C6="",0,IF(YEAR($C6)=$B$3,1,0))</f>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="Y6">
-        <f>IF($C6="",0,IF(AND($I6&lt;&gt;"",YEAR($I6)=$B$3),1,0))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" s="5" t="s">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="Z6" s="13" t="str">
+        <f>IF($C6="","",IF($F6&lt;=0,"Life must be greater than 0",IF($D6&lt;0,"Cost cannot be negative",IF($E6&gt;$D6,"Salvage exceeds cost",IF(YEAR($C6)&gt;$B$3,"In-service date is after the report year",IF(AND($I6&lt;&gt;"",$I6&lt;$C6),"Disposal date is before in-service date",IF(ISNA(MATCH($G6,Tables!$B$2:$F$2,0)),"Tax class must be 3, 5, 7, 10 or 15",IF($AA6=1,"Disposed in a prior year - remove this row","OK"))))))))</f>
+        <v>OK</v>
+      </c>
+      <c r="AA6" s="4">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>35</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>36</v>
       </c>
       <c r="C7" s="6">
         <v>46042</v>
@@ -1242,84 +1407,92 @@
       <c r="E7" s="7">
         <v>0</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="4">
         <v>3</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="4">
         <v>5</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H7" s="8">
         <v>0.8</v>
       </c>
       <c r="I7" s="6"/>
       <c r="J7" s="7"/>
       <c r="K7">
-        <f>IF($C7="","",MAX(0,MIN($F7*12,($B$3-1-YEAR($C7))*12+13-MONTH($C7))))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L7">
-        <f>IF($C7="","",IF(YEAR($C7)&gt;$B$3,0,IF(AND($I7&lt;&gt;"",YEAR($I7)&lt;$B$3),0,MAX(0,MIN(IF(AND($I7&lt;&gt;"",YEAR($I7)=$B$3),MONTH($I7)-1,12)-IF(YEAR($C7)=$B$3,MONTH($C7),1)+1,$F7*12-K7)))))</f>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="M7" s="9">
-        <f>IF($C7="","",($D7-$E7)/($F7*12))</f>
+        <f t="shared" si="2"/>
         <v>248.33333333333334</v>
       </c>
       <c r="N7" s="9">
-        <f>IF($C7="","",K7*M7)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O7" s="9">
-        <f>IF($C7="","",L7*M7)</f>
+        <f t="shared" si="4"/>
         <v>2980</v>
       </c>
       <c r="P7" s="9">
-        <f>IF(Y7=1,N7+O7,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Q7" s="9">
-        <f>IF($C7="","",IF(Y7=1,0,N7+O7))</f>
+        <f t="shared" si="6"/>
         <v>2980</v>
       </c>
       <c r="R7" s="9">
-        <f>IF($C7="","",IF(OR(Y7=1,AND($I7&lt;&gt;"",YEAR($I7)&lt;$B$3)),0,$D7))</f>
+        <f t="shared" si="7"/>
         <v>8940</v>
       </c>
       <c r="S7" s="9">
-        <f>IF($C7="","",R7-Q7)</f>
+        <f t="shared" si="8"/>
         <v>5960</v>
       </c>
       <c r="T7" s="9" t="str">
-        <f>IF(Y7=1,$J7-($D7-P7),"")</f>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="U7">
-        <f>IF($C7="","",$B$3-YEAR($C7)+1)</f>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
-      <c r="V7" s="1" cm="1">
-        <f t="array" ref="V7">IF($C7="","",IFERROR(INDEX(Tables!$B$3:$F$18,U7,MATCH($G7,Tables!$B$2:$F$2,0)),0))</f>
+      <c r="V7" s="1">
+        <f>IF($C7="","",IF(U7&lt;1,0,IFERROR(INDEX(Tables!$B$3:$F$18,U7,MATCH($G7,Tables!$B$2:$F$2,0)),0)))</f>
         <v>0.2</v>
       </c>
       <c r="W7" s="9">
-        <f>IF($C7="","",IF(AND($I7&lt;&gt;"",YEAR($I7)&lt;$B$3),0,($D7*(1-$H7))*V7*IF(Y7=1,0.5,1)+IF(U7=1,$D7*$H7,0)))</f>
+        <f t="shared" si="11"/>
         <v>7509.6</v>
       </c>
       <c r="X7">
-        <f>IF($C7="",0,IF(YEAR($C7)=$B$3,1,0))</f>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="Y7">
-        <f>IF($C7="",0,IF(AND($I7&lt;&gt;"",YEAR($I7)=$B$3),1,0))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="B8" s="5" t="s">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="Z7" s="13" t="str">
+        <f>IF($C7="","",IF($F7&lt;=0,"Life must be greater than 0",IF($D7&lt;0,"Cost cannot be negative",IF($E7&gt;$D7,"Salvage exceeds cost",IF(YEAR($C7)&gt;$B$3,"In-service date is after the report year",IF(AND($I7&lt;&gt;"",$I7&lt;$C7),"Disposal date is before in-service date",IF(ISNA(MATCH($G7,Tables!$B$2:$F$2,0)),"Tax class must be 3, 5, 7, 10 or 15",IF($AA7=1,"Disposed in a prior year - remove this row","OK"))))))))</f>
+        <v>OK</v>
+      </c>
+      <c r="AA7" s="4">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>37</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>38</v>
       </c>
       <c r="C8" s="6">
         <v>46122</v>
@@ -1330,84 +1503,92 @@
       <c r="E8" s="7">
         <v>4800</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="4">
         <v>5</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="4">
         <v>5</v>
       </c>
-      <c r="H8" s="10">
+      <c r="H8" s="8">
         <v>0</v>
       </c>
       <c r="I8" s="6"/>
       <c r="J8" s="7"/>
       <c r="K8">
-        <f>IF($C8="","",MAX(0,MIN($F8*12,($B$3-1-YEAR($C8))*12+13-MONTH($C8))))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L8">
-        <f>IF($C8="","",IF(YEAR($C8)&gt;$B$3,0,IF(AND($I8&lt;&gt;"",YEAR($I8)&lt;$B$3),0,MAX(0,MIN(IF(AND($I8&lt;&gt;"",YEAR($I8)=$B$3),MONTH($I8)-1,12)-IF(YEAR($C8)=$B$3,MONTH($C8),1)+1,$F8*12-K8)))))</f>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="M8" s="9">
-        <f>IF($C8="","",($D8-$E8)/($F8*12))</f>
+        <f t="shared" si="2"/>
         <v>800</v>
       </c>
       <c r="N8" s="9">
-        <f>IF($C8="","",K8*M8)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O8" s="9">
-        <f>IF($C8="","",L8*M8)</f>
+        <f t="shared" si="4"/>
         <v>7200</v>
       </c>
       <c r="P8" s="9">
-        <f>IF(Y8=1,N8+O8,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Q8" s="9">
-        <f>IF($C8="","",IF(Y8=1,0,N8+O8))</f>
+        <f t="shared" si="6"/>
         <v>7200</v>
       </c>
       <c r="R8" s="9">
-        <f>IF($C8="","",IF(OR(Y8=1,AND($I8&lt;&gt;"",YEAR($I8)&lt;$B$3)),0,$D8))</f>
+        <f t="shared" si="7"/>
         <v>52800</v>
       </c>
       <c r="S8" s="9">
-        <f>IF($C8="","",R8-Q8)</f>
+        <f t="shared" si="8"/>
         <v>45600</v>
       </c>
       <c r="T8" s="9" t="str">
-        <f>IF(Y8=1,$J8-($D8-P8),"")</f>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="U8">
-        <f>IF($C8="","",$B$3-YEAR($C8)+1)</f>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
-      <c r="V8" s="1" cm="1">
-        <f t="array" ref="V8">IF($C8="","",IFERROR(INDEX(Tables!$B$3:$F$18,U8,MATCH($G8,Tables!$B$2:$F$2,0)),0))</f>
+      <c r="V8" s="1">
+        <f>IF($C8="","",IF(U8&lt;1,0,IFERROR(INDEX(Tables!$B$3:$F$18,U8,MATCH($G8,Tables!$B$2:$F$2,0)),0)))</f>
         <v>0.2</v>
       </c>
       <c r="W8" s="9">
-        <f>IF($C8="","",IF(AND($I8&lt;&gt;"",YEAR($I8)&lt;$B$3),0,($D8*(1-$H8))*V8*IF(Y8=1,0.5,1)+IF(U8=1,$D8*$H8,0)))</f>
+        <f t="shared" si="11"/>
         <v>10560</v>
       </c>
       <c r="X8">
-        <f>IF($C8="",0,IF(YEAR($C8)=$B$3,1,0))</f>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="Y8">
-        <f>IF($C8="",0,IF(AND($I8&lt;&gt;"",YEAR($I8)=$B$3),1,0))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B9" s="5" t="s">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="Z8" s="13" t="str">
+        <f>IF($C8="","",IF($F8&lt;=0,"Life must be greater than 0",IF($D8&lt;0,"Cost cannot be negative",IF($E8&gt;$D8,"Salvage exceeds cost",IF(YEAR($C8)&gt;$B$3,"In-service date is after the report year",IF(AND($I8&lt;&gt;"",$I8&lt;$C8),"Disposal date is before in-service date",IF(ISNA(MATCH($G8,Tables!$B$2:$F$2,0)),"Tax class must be 3, 5, 7, 10 or 15",IF($AA8=1,"Disposed in a prior year - remove this row","OK"))))))))</f>
+        <v>OK</v>
+      </c>
+      <c r="AA8" s="4">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>39</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="C9" s="6">
         <v>44440</v>
@@ -1418,84 +1599,92 @@
       <c r="E9" s="7">
         <v>5000</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="4">
         <v>10</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="4">
         <v>7</v>
       </c>
-      <c r="H9" s="10">
+      <c r="H9" s="8">
         <v>0</v>
       </c>
       <c r="I9" s="6"/>
       <c r="J9" s="7"/>
       <c r="K9">
-        <f>IF($C9="","",MAX(0,MIN($F9*12,($B$3-1-YEAR($C9))*12+13-MONTH($C9))))</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
       <c r="L9">
-        <f>IF($C9="","",IF(YEAR($C9)&gt;$B$3,0,IF(AND($I9&lt;&gt;"",YEAR($I9)&lt;$B$3),0,MAX(0,MIN(IF(AND($I9&lt;&gt;"",YEAR($I9)=$B$3),MONTH($I9)-1,12)-IF(YEAR($C9)=$B$3,MONTH($C9),1)+1,$F9*12-K9)))))</f>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="M9" s="9">
-        <f>IF($C9="","",($D9-$E9)/($F9*12))</f>
+        <f t="shared" si="2"/>
         <v>1166.6666666666667</v>
       </c>
       <c r="N9" s="9">
-        <f>IF($C9="","",K9*M9)</f>
+        <f t="shared" si="3"/>
         <v>60666.666666666672</v>
       </c>
       <c r="O9" s="9">
-        <f>IF($C9="","",L9*M9)</f>
+        <f t="shared" si="4"/>
         <v>14000</v>
       </c>
       <c r="P9" s="9">
-        <f>IF(Y9=1,N9+O9,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Q9" s="9">
-        <f>IF($C9="","",IF(Y9=1,0,N9+O9))</f>
+        <f t="shared" si="6"/>
         <v>74666.666666666672</v>
       </c>
       <c r="R9" s="9">
-        <f>IF($C9="","",IF(OR(Y9=1,AND($I9&lt;&gt;"",YEAR($I9)&lt;$B$3)),0,$D9))</f>
+        <f t="shared" si="7"/>
         <v>145000</v>
       </c>
       <c r="S9" s="9">
-        <f>IF($C9="","",R9-Q9)</f>
+        <f t="shared" si="8"/>
         <v>70333.333333333328</v>
       </c>
       <c r="T9" s="9" t="str">
-        <f>IF(Y9=1,$J9-($D9-P9),"")</f>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="U9">
-        <f>IF($C9="","",$B$3-YEAR($C9)+1)</f>
+        <f t="shared" si="10"/>
         <v>6</v>
       </c>
-      <c r="V9" s="1" cm="1">
-        <f t="array" ref="V9">IF($C9="","",IFERROR(INDEX(Tables!$B$3:$F$18,U9,MATCH($G9,Tables!$B$2:$F$2,0)),0))</f>
+      <c r="V9" s="1">
+        <f>IF($C9="","",IF(U9&lt;1,0,IFERROR(INDEX(Tables!$B$3:$F$18,U9,MATCH($G9,Tables!$B$2:$F$2,0)),0)))</f>
         <v>8.9200000000000002E-2</v>
       </c>
       <c r="W9" s="9">
-        <f>IF($C9="","",IF(AND($I9&lt;&gt;"",YEAR($I9)&lt;$B$3),0,($D9*(1-$H9))*V9*IF(Y9=1,0.5,1)+IF(U9=1,$D9*$H9,0)))</f>
+        <f t="shared" si="11"/>
         <v>12934</v>
       </c>
       <c r="X9">
-        <f>IF($C9="",0,IF(YEAR($C9)=$B$3,1,0))</f>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="Y9">
-        <f>IF($C9="",0,IF(AND($I9&lt;&gt;"",YEAR($I9)=$B$3),1,0))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B10" s="5" t="s">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="Z9" s="13" t="str">
+        <f>IF($C9="","",IF($F9&lt;=0,"Life must be greater than 0",IF($D9&lt;0,"Cost cannot be negative",IF($E9&gt;$D9,"Salvage exceeds cost",IF(YEAR($C9)&gt;$B$3,"In-service date is after the report year",IF(AND($I9&lt;&gt;"",$I9&lt;$C9),"Disposal date is before in-service date",IF(ISNA(MATCH($G9,Tables!$B$2:$F$2,0)),"Tax class must be 3, 5, 7, 10 or 15",IF($AA9=1,"Disposed in a prior year - remove this row","OK"))))))))</f>
+        <v>OK</v>
+      </c>
+      <c r="AA9" s="4">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>41</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="C10" s="6">
         <v>44693</v>
@@ -1506,13 +1695,13 @@
       <c r="E10" s="7">
         <v>0</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="4">
         <v>5</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="4">
         <v>5</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10" s="8">
         <v>0</v>
       </c>
       <c r="I10" s="6">
@@ -1522,123 +1711,138 @@
         <v>4200</v>
       </c>
       <c r="K10">
-        <f>IF($C10="","",MAX(0,MIN($F10*12,($B$3-1-YEAR($C10))*12+13-MONTH($C10))))</f>
+        <f t="shared" si="0"/>
         <v>44</v>
       </c>
       <c r="L10">
-        <f>IF($C10="","",IF(YEAR($C10)&gt;$B$3,0,IF(AND($I10&lt;&gt;"",YEAR($I10)&lt;$B$3),0,MAX(0,MIN(IF(AND($I10&lt;&gt;"",YEAR($I10)=$B$3),MONTH($I10)-1,12)-IF(YEAR($C10)=$B$3,MONTH($C10),1)+1,$F10*12-K10)))))</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="M10" s="9">
-        <f>IF($C10="","",($D10-$E10)/($F10*12))</f>
+        <f t="shared" si="2"/>
         <v>310</v>
       </c>
       <c r="N10" s="9">
-        <f>IF($C10="","",K10*M10)</f>
+        <f t="shared" si="3"/>
         <v>13640</v>
       </c>
       <c r="O10" s="9">
-        <f>IF($C10="","",L10*M10)</f>
+        <f t="shared" si="4"/>
         <v>1550</v>
       </c>
       <c r="P10" s="9">
-        <f>IF(Y10=1,N10+O10,0)</f>
+        <f t="shared" si="5"/>
         <v>15190</v>
       </c>
       <c r="Q10" s="9">
-        <f>IF($C10="","",IF(Y10=1,0,N10+O10))</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="R10" s="9">
-        <f>IF($C10="","",IF(OR(Y10=1,AND($I10&lt;&gt;"",YEAR($I10)&lt;$B$3)),0,$D10))</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="S10" s="9">
-        <f>IF($C10="","",R10-Q10)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="T10" s="9">
-        <f>IF(Y10=1,$J10-($D10-P10),"")</f>
+        <f t="shared" si="9"/>
         <v>790</v>
       </c>
       <c r="U10">
-        <f>IF($C10="","",$B$3-YEAR($C10)+1)</f>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
-      <c r="V10" s="1" cm="1">
-        <f t="array" ref="V10">IF($C10="","",IFERROR(INDEX(Tables!$B$3:$F$18,U10,MATCH($G10,Tables!$B$2:$F$2,0)),0))</f>
+      <c r="V10" s="1">
+        <f>IF($C10="","",IF(U10&lt;1,0,IFERROR(INDEX(Tables!$B$3:$F$18,U10,MATCH($G10,Tables!$B$2:$F$2,0)),0)))</f>
         <v>0.1152</v>
       </c>
       <c r="W10" s="9">
-        <f>IF($C10="","",IF(AND($I10&lt;&gt;"",YEAR($I10)&lt;$B$3),0,($D10*(1-$H10))*V10*IF(Y10=1,0.5,1)+IF(U10=1,$D10*$H10,0)))</f>
+        <f t="shared" si="11"/>
         <v>1071.3599999999999</v>
       </c>
       <c r="X10">
-        <f>IF($C10="",0,IF(YEAR($C10)=$B$3,1,0))</f>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="Y10">
-        <f>IF($C10="",0,IF(AND($I10&lt;&gt;"",YEAR($I10)=$B$3),1,0))</f>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B11" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" s="8">
+      <c r="Z10" s="13" t="str">
+        <f>IF($C10="","",IF($F10&lt;=0,"Life must be greater than 0",IF($D10&lt;0,"Cost cannot be negative",IF($E10&gt;$D10,"Salvage exceeds cost",IF(YEAR($C10)&gt;$B$3,"In-service date is after the report year",IF(AND($I10&lt;&gt;"",$I10&lt;$C10),"Disposal date is before in-service date",IF(ISNA(MATCH($G10,Tables!$B$2:$F$2,0)),"Tax class must be 3, 5, 7, 10 or 15",IF($AA10=1,"Disposed in a prior year - remove this row","OK"))))))))</f>
+        <v>OK</v>
+      </c>
+      <c r="AA10" s="4">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="10">
         <f>SUM(D5:D10)</f>
         <v>318040</v>
       </c>
       <c r="E11" s="9"/>
+      <c r="J11" s="10">
+        <f>SUM(J5:J10)</f>
+        <v>4200</v>
+      </c>
       <c r="M11" s="9"/>
-      <c r="N11" s="8">
-        <f>SUM(N5:N10)</f>
+      <c r="N11" s="10">
+        <f t="shared" ref="N11:T11" si="15">SUM(N5:N10)</f>
         <v>94460.476190476198</v>
       </c>
-      <c r="O11" s="8">
-        <f>SUM(O5:O10)</f>
+      <c r="O11" s="10">
+        <f t="shared" si="15"/>
         <v>35864.28571428571</v>
       </c>
-      <c r="P11" s="8">
-        <f>SUM(P5:P10)</f>
+      <c r="P11" s="10">
+        <f t="shared" si="15"/>
         <v>15190</v>
       </c>
-      <c r="Q11" s="8">
-        <f>SUM(Q5:Q10)</f>
+      <c r="Q11" s="10">
+        <f t="shared" si="15"/>
         <v>115134.76190476191</v>
       </c>
-      <c r="R11" s="8">
-        <f>SUM(R5:R10)</f>
+      <c r="R11" s="10">
+        <f t="shared" si="15"/>
         <v>299440</v>
       </c>
-      <c r="S11" s="8">
-        <f>SUM(S5:S10)</f>
+      <c r="S11" s="10">
+        <f t="shared" si="15"/>
         <v>184305.23809523811</v>
       </c>
-      <c r="T11" s="9"/>
-      <c r="W11" s="8">
+      <c r="T11" s="10">
+        <f t="shared" si="15"/>
+        <v>790</v>
+      </c>
+      <c r="W11" s="10">
         <f>SUM(W5:W10)</f>
         <v>40847.26</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>43</v>
+    <row r="14" spans="1:27" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>45</v>
-      </c>
-      <c r="B15" s="9" cm="1">
-        <f t="array" ref="B15">SUMPRODUCT(($C$5:$C$10&lt;&gt;"")*(1-$X$5:$X$10)*$D$5:$D$10)</f>
+        <v>46</v>
+      </c>
+      <c r="B15" s="9">
+        <f>SUMPRODUCT(($C$5:$C$10&lt;&gt;"")*(1-$X$5:$X$10)*(1-$AA$5:$AA$10)*$D$5:$D$10)</f>
         <v>256300</v>
       </c>
       <c r="C15" s="9">
@@ -1646,12 +1850,12 @@
         <v>94460.476190476198</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16" s="9" cm="1">
-        <f t="array" ref="B16">SUMPRODUCT($X$5:$X$10*$D$5:$D$10)</f>
+        <v>47</v>
+      </c>
+      <c r="B16" s="9">
+        <f>SUMPRODUCT($X$5:$X$10*$D$5:$D$10)</f>
         <v>61740</v>
       </c>
       <c r="C16" s="9">
@@ -1659,12 +1863,12 @@
         <v>35864.28571428571</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>47</v>
-      </c>
-      <c r="B17" s="9" cm="1">
-        <f t="array" ref="B17">-SUMPRODUCT($Y$5:$Y$10*$D$5:$D$10)</f>
+        <v>48</v>
+      </c>
+      <c r="B17" s="9">
+        <f>-SUMPRODUCT($Y$5:$Y$10*$D$5:$D$10)</f>
         <v>-18600</v>
       </c>
       <c r="C17" s="9">
@@ -1672,22 +1876,22 @@
         <v>-15190</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" s="8">
+        <v>49</v>
+      </c>
+      <c r="B18" s="10">
         <f>SUM(B15:B17)</f>
         <v>299440</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="10">
         <f>SUM(C15:C17)</f>
         <v>115134.76190476191</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B19" s="9" t="str">
         <f>IF(ROUND(B18-$R$11,2)=0,"OK",B18-$R$11)</f>
@@ -1698,19 +1902,19 @@
         <v>OK</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>50</v>
-      </c>
-      <c r="B20" s="8">
+        <v>51</v>
+      </c>
+      <c r="B20" s="10">
         <f>B18-C18</f>
         <v>184305.23809523811</v>
       </c>
       <c r="C20" s="9"/>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B21" s="9" t="str">
         <f>IF(ROUND(B20-$S$11,2)=0,"OK",B20-$S$11)</f>
@@ -1718,14 +1922,23 @@
       </c>
       <c r="C21" s="9"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="9" t="str">
+        <f>IF(SUMPRODUCT(($C$5:$C$10&lt;&gt;"")*($Z$5:$Z$10&lt;&gt;"OK"))=0,"OK",SUMPRODUCT(($C$5:$C$10&lt;&gt;"")*($Z$5:$Z$10&lt;&gt;"OK"))&amp;" row(s) need attention - see Check column")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" t="str">
@@ -1733,9 +1946,9 @@
         <v>enter GL balance</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" t="str">
@@ -1744,64 +1957,79 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{708753D3-2D79-437A-881D-171276B0DF9E}">
-  <dimension ref="A1:A10"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:A12"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="110.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>62</v>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>